<commit_message>
fix: remove sample rows from PO and Master SKU templates
Sample row on row 4 would be parsed as real data on upload.
Templates now have only 3 rows: title, instructions, headers.
User fills data from row 4 onward.
</commit_message>
<xml_diff>
--- a/public/templates/CTG_Master_SKU_Template.xlsx
+++ b/public/templates/CTG_Master_SKU_Template.xlsx
@@ -460,7 +460,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L4"/>
+  <dimension ref="A1:L3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -553,50 +553,7 @@
         </is>
       </c>
     </row>
-    <row r="4" ht="18" customHeight="1">
-      <c r="A4" s="4" t="inlineStr">
-        <is>
-          <t>SDSDCA030</t>
-        </is>
-      </c>
-      <c r="B4" s="4" t="inlineStr">
-        <is>
-          <t>SkinDae</t>
-        </is>
-      </c>
-      <c r="C4" s="4" t="inlineStr">
-        <is>
-          <t>SkinDae, Cell Lift Ampoule, 30ml</t>
-        </is>
-      </c>
-      <c r="D4" s="4" t="inlineStr">
-        <is>
-          <t>Bottle</t>
-        </is>
-      </c>
-      <c r="E4" s="4" t="n">
-        <v>10000</v>
-      </c>
-      <c r="F4" s="4" t="n">
-        <v>11</v>
-      </c>
-      <c r="G4" s="4" t="n">
-        <v>190</v>
-      </c>
-      <c r="H4" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="I4" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="J4" s="4" t="inlineStr">
-        <is>
-          <t>Active</t>
-        </is>
-      </c>
-      <c r="K4" s="4" t="inlineStr"/>
-      <c r="L4" s="4" t="inlineStr"/>
-    </row>
+    <row r="4" ht="18" customHeight="1"/>
   </sheetData>
   <mergeCells count="2">
     <mergeCell ref="A2:L2"/>

</xml_diff>